<commit_message>
Power Blocs for Isolationism, Luxury Textile Mill, Rayon Focus
</commit_message>
<xml_diff>
--- a/IndustryExpanded/FACTORIES.xlsx
+++ b/IndustryExpanded/FACTORIES.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3TO_9I\Documents\Paradox Interactive\Victoria 3\mod\IndustryExpanded\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED96DE1E-DDAB-4382-A81D-3FD4DCE7E188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9163B363-C92C-4AA2-BD35-39D493A8DBAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{E8AEE59E-FFCD-4A72-B877-FD5D3ADEE5A1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="78">
   <si>
     <t>Building</t>
   </si>
@@ -255,6 +255,21 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>Logging Camps</t>
+  </si>
+  <si>
+    <t>Backwards</t>
+  </si>
+  <si>
+    <t>Tools</t>
+  </si>
+  <si>
+    <t>Tools, Steam Donkey, Rail</t>
+  </si>
+  <si>
+    <t>Electric, Chainsaws, Carts</t>
   </si>
 </sst>
 </file>
@@ -551,6 +566,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -559,9 +577,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -905,7 +920,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{619B0D70-D2AF-46B3-9D3D-17ECB8467BBA}">
-  <dimension ref="A1:N131"/>
+  <dimension ref="A1:N148"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -958,7 +973,7 @@
       <c r="E2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="33" t="s">
+      <c r="F2" s="30" t="s">
         <v>8</v>
       </c>
       <c r="G2" s="14">
@@ -980,7 +995,7 @@
       <c r="M2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="N2" s="33" t="s">
+      <c r="N2" s="30" t="s">
         <v>13</v>
       </c>
     </row>
@@ -996,7 +1011,7 @@
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="9"/>
-      <c r="F3" s="33"/>
+      <c r="F3" s="30"/>
       <c r="G3" s="16">
         <v>1200</v>
       </c>
@@ -1013,7 +1028,7 @@
       </c>
       <c r="L3" s="3"/>
       <c r="M3" s="9"/>
-      <c r="N3" s="33"/>
+      <c r="N3" s="30"/>
     </row>
     <row r="4" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
@@ -1033,7 +1048,7 @@
       <c r="E4" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="33"/>
+      <c r="F4" s="30"/>
       <c r="G4" s="15">
         <f>G3-G2</f>
         <v>600</v>
@@ -1058,7 +1073,7 @@
       <c r="M4" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="N4" s="33"/>
+      <c r="N4" s="30"/>
     </row>
     <row r="5" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
@@ -1077,7 +1092,7 @@
       <c r="E5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="33" t="s">
+      <c r="F5" s="30" t="s">
         <v>9</v>
       </c>
       <c r="G5" s="14">
@@ -1100,7 +1115,7 @@
       <c r="M5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="N5" s="33" t="s">
+      <c r="N5" s="30" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1117,7 +1132,7 @@
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="9"/>
-      <c r="F6" s="33"/>
+      <c r="F6" s="30"/>
       <c r="G6" s="16">
         <v>2400</v>
       </c>
@@ -1133,7 +1148,7 @@
       </c>
       <c r="L6" s="3"/>
       <c r="M6" s="9"/>
-      <c r="N6" s="33"/>
+      <c r="N6" s="30"/>
     </row>
     <row r="7" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
@@ -1153,7 +1168,7 @@
       <c r="E7" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F7" s="33"/>
+      <c r="F7" s="30"/>
       <c r="G7" s="15">
         <f>G6-G5</f>
         <v>800</v>
@@ -1178,7 +1193,7 @@
       <c r="M7" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="N7" s="33"/>
+      <c r="N7" s="30"/>
     </row>
     <row r="8" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
@@ -1197,7 +1212,7 @@
       <c r="E8" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F8" s="33" t="s">
+      <c r="F8" s="30" t="s">
         <v>10</v>
       </c>
       <c r="G8" s="14">
@@ -1220,7 +1235,7 @@
       <c r="M8" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="N8" s="33" t="s">
+      <c r="N8" s="30" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1237,7 +1252,7 @@
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="9"/>
-      <c r="F9" s="33"/>
+      <c r="F9" s="30"/>
       <c r="G9" s="16">
         <v>3200</v>
       </c>
@@ -1254,7 +1269,7 @@
       </c>
       <c r="L9" s="3"/>
       <c r="M9" s="9"/>
-      <c r="N9" s="33"/>
+      <c r="N9" s="30"/>
     </row>
     <row r="10" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
@@ -1274,7 +1289,7 @@
       <c r="E10" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F10" s="33"/>
+      <c r="F10" s="30"/>
       <c r="G10" s="15">
         <f>G9-G8</f>
         <v>1100</v>
@@ -1299,7 +1314,7 @@
       <c r="M10" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="N10" s="33"/>
+      <c r="N10" s="30"/>
     </row>
     <row r="11" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
@@ -1318,7 +1333,7 @@
       <c r="E11" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F11" s="33" t="s">
+      <c r="F11" s="30" t="s">
         <v>11</v>
       </c>
       <c r="G11" s="14">
@@ -1341,7 +1356,7 @@
       <c r="M11" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="N11" s="33" t="s">
+      <c r="N11" s="30" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1358,7 +1373,7 @@
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="9"/>
-      <c r="F12" s="33"/>
+      <c r="F12" s="30"/>
       <c r="G12" s="16">
         <v>4200</v>
       </c>
@@ -1375,7 +1390,7 @@
       </c>
       <c r="L12" s="3"/>
       <c r="M12" s="9"/>
-      <c r="N12" s="33"/>
+      <c r="N12" s="30"/>
     </row>
     <row r="13" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
@@ -1395,7 +1410,7 @@
       <c r="E13" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F13" s="33"/>
+      <c r="F13" s="30"/>
       <c r="G13" s="15">
         <f>G12-G11</f>
         <v>1800</v>
@@ -1420,7 +1435,7 @@
       <c r="M13" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="N13" s="33"/>
+      <c r="N13" s="30"/>
     </row>
     <row r="14" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
@@ -1456,7 +1471,7 @@
       <c r="E15" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F15" s="33" t="s">
+      <c r="F15" s="30" t="s">
         <v>26</v>
       </c>
       <c r="G15" s="14">
@@ -1492,7 +1507,7 @@
       </c>
       <c r="D16" s="3"/>
       <c r="E16" s="9"/>
-      <c r="F16" s="33"/>
+      <c r="F16" s="30"/>
       <c r="G16" s="16">
         <v>1200</v>
       </c>
@@ -1527,7 +1542,7 @@
       <c r="E17" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F17" s="33"/>
+      <c r="F17" s="30"/>
       <c r="G17" s="15">
         <f>G16-G15</f>
         <v>600</v>
@@ -1569,7 +1584,7 @@
       <c r="E18" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F18" s="33" t="s">
+      <c r="F18" s="30" t="s">
         <v>25</v>
       </c>
       <c r="G18" s="14">
@@ -1606,7 +1621,7 @@
       </c>
       <c r="D19" s="3"/>
       <c r="E19" s="9"/>
-      <c r="F19" s="33"/>
+      <c r="F19" s="30"/>
       <c r="G19" s="16">
         <v>2400</v>
       </c>
@@ -1642,7 +1657,7 @@
       <c r="E20" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F20" s="33"/>
+      <c r="F20" s="30"/>
       <c r="G20" s="15">
         <f>G19-G18</f>
         <v>800</v>
@@ -1776,7 +1791,7 @@
       <c r="E24" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F24" s="33" t="s">
+      <c r="F24" s="30" t="s">
         <v>27</v>
       </c>
       <c r="G24" s="14">
@@ -1805,7 +1820,7 @@
       </c>
       <c r="D25" s="3"/>
       <c r="E25" s="9"/>
-      <c r="F25" s="33"/>
+      <c r="F25" s="30"/>
       <c r="G25" s="16">
         <v>4200</v>
       </c>
@@ -1835,7 +1850,7 @@
       <c r="E26" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F26" s="33"/>
+      <c r="F26" s="30"/>
       <c r="G26" s="15">
         <f>G25-G24</f>
         <v>1800</v>
@@ -1904,7 +1919,7 @@
       <c r="E31" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F31" s="33" t="s">
+      <c r="F31" s="30" t="s">
         <v>29</v>
       </c>
       <c r="G31" s="14">
@@ -1921,7 +1936,7 @@
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="9"/>
-      <c r="F32" s="33"/>
+      <c r="F32" s="30"/>
       <c r="G32" s="16">
         <v>2400</v>
       </c>
@@ -1943,7 +1958,7 @@
       <c r="E33" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F33" s="33"/>
+      <c r="F33" s="30"/>
       <c r="G33" s="15">
         <f>G32-G31</f>
         <v>800</v>
@@ -2097,7 +2112,7 @@
       <c r="A41" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B41" s="30" t="s">
+      <c r="B41" s="31" t="s">
         <v>32</v>
       </c>
       <c r="C41" s="6">
@@ -2109,7 +2124,7 @@
       <c r="E41" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F41" s="33" t="s">
+      <c r="F41" s="30" t="s">
         <v>33</v>
       </c>
       <c r="G41" s="14">
@@ -2121,13 +2136,13 @@
       <c r="A42" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B42" s="31"/>
+      <c r="B42" s="32"/>
       <c r="C42" s="3">
         <v>1200</v>
       </c>
       <c r="D42" s="3"/>
       <c r="E42" s="9"/>
-      <c r="F42" s="33"/>
+      <c r="F42" s="30"/>
       <c r="G42" s="16">
         <v>1200</v>
       </c>
@@ -2137,7 +2152,7 @@
       <c r="A43" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B43" s="32"/>
+      <c r="B43" s="33"/>
       <c r="C43" s="12">
         <f>C42-C41</f>
         <v>540</v>
@@ -2149,7 +2164,7 @@
       <c r="E43" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F43" s="33"/>
+      <c r="F43" s="30"/>
       <c r="G43" s="15">
         <f>G42-G41</f>
         <v>600</v>
@@ -2162,7 +2177,7 @@
       <c r="A44" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B44" s="30" t="s">
+      <c r="B44" s="31" t="s">
         <v>32</v>
       </c>
       <c r="C44" s="6">
@@ -2174,7 +2189,7 @@
       <c r="E44" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F44" s="33" t="s">
+      <c r="F44" s="30" t="s">
         <v>41</v>
       </c>
       <c r="G44" s="14">
@@ -2186,13 +2201,13 @@
       <c r="A45" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B45" s="31"/>
+      <c r="B45" s="32"/>
       <c r="C45" s="3">
         <v>2010</v>
       </c>
       <c r="D45" s="3"/>
       <c r="E45" s="9"/>
-      <c r="F45" s="33"/>
+      <c r="F45" s="30"/>
       <c r="G45" s="16">
         <v>2000</v>
       </c>
@@ -2202,7 +2217,7 @@
       <c r="A46" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B46" s="32"/>
+      <c r="B46" s="33"/>
       <c r="C46" s="12">
         <f>C45-C44</f>
         <v>810</v>
@@ -2214,7 +2229,7 @@
       <c r="E46" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F46" s="33"/>
+      <c r="F46" s="30"/>
       <c r="G46" s="15">
         <f>G45-G44</f>
         <v>800</v>
@@ -2227,7 +2242,7 @@
       <c r="A47" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B47" s="30" t="s">
+      <c r="B47" s="31" t="s">
         <v>32</v>
       </c>
       <c r="C47" s="20">
@@ -2239,7 +2254,7 @@
       <c r="E47" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F47" s="33" t="s">
+      <c r="F47" s="30" t="s">
         <v>40</v>
       </c>
       <c r="G47" s="14">
@@ -2251,13 +2266,13 @@
       <c r="A48" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B48" s="31"/>
+      <c r="B48" s="32"/>
       <c r="C48" s="20">
         <v>2880</v>
       </c>
       <c r="D48" s="20"/>
       <c r="E48" s="9"/>
-      <c r="F48" s="33"/>
+      <c r="F48" s="30"/>
       <c r="G48" s="16">
         <v>2900</v>
       </c>
@@ -2267,7 +2282,7 @@
       <c r="A49" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B49" s="32"/>
+      <c r="B49" s="33"/>
       <c r="C49" s="12">
         <f>C48-C47</f>
         <v>1080</v>
@@ -2279,7 +2294,7 @@
       <c r="E49" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F49" s="33"/>
+      <c r="F49" s="30"/>
       <c r="G49" s="15">
         <f>G48-G47</f>
         <v>1100</v>
@@ -2292,7 +2307,7 @@
       <c r="A50" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B50" s="30" t="s">
+      <c r="B50" s="31" t="s">
         <v>32</v>
       </c>
       <c r="C50" s="6">
@@ -2304,7 +2319,7 @@
       <c r="E50" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F50" s="33" t="s">
+      <c r="F50" s="30" t="s">
         <v>39</v>
       </c>
       <c r="G50" s="14">
@@ -2316,13 +2331,13 @@
       <c r="A51" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B51" s="31"/>
+      <c r="B51" s="32"/>
       <c r="C51" s="3">
         <v>4200</v>
       </c>
       <c r="D51" s="3"/>
       <c r="E51" s="9"/>
-      <c r="F51" s="33"/>
+      <c r="F51" s="30"/>
       <c r="G51" s="16">
         <v>4200</v>
       </c>
@@ -2332,7 +2347,7 @@
       <c r="A52" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B52" s="32"/>
+      <c r="B52" s="33"/>
       <c r="C52" s="12">
         <f>C51-C50</f>
         <v>1800</v>
@@ -2344,7 +2359,7 @@
       <c r="E52" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F52" s="33"/>
+      <c r="F52" s="30"/>
       <c r="G52" s="15">
         <f>G51-G50</f>
         <v>1800</v>
@@ -2371,7 +2386,7 @@
       <c r="A54" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B54" s="30" t="s">
+      <c r="B54" s="31" t="s">
         <v>34</v>
       </c>
       <c r="C54" s="6">
@@ -2383,7 +2398,7 @@
       <c r="E54" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F54" s="33" t="s">
+      <c r="F54" s="30" t="s">
         <v>35</v>
       </c>
       <c r="G54" s="14">
@@ -2395,13 +2410,13 @@
       <c r="A55" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B55" s="31"/>
+      <c r="B55" s="32"/>
       <c r="C55" s="3">
         <v>1200</v>
       </c>
       <c r="D55" s="3"/>
       <c r="E55" s="9"/>
-      <c r="F55" s="33"/>
+      <c r="F55" s="30"/>
       <c r="G55" s="16">
         <v>1200</v>
       </c>
@@ -2411,7 +2426,7 @@
       <c r="A56" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B56" s="32"/>
+      <c r="B56" s="33"/>
       <c r="C56" s="12">
         <f>C55-C54</f>
         <v>600</v>
@@ -2423,7 +2438,7 @@
       <c r="E56" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F56" s="33"/>
+      <c r="F56" s="30"/>
       <c r="G56" s="15">
         <f>G55-G54</f>
         <v>600</v>
@@ -2436,7 +2451,7 @@
       <c r="A57" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B57" s="30" t="s">
+      <c r="B57" s="31" t="s">
         <v>34</v>
       </c>
       <c r="C57" s="6">
@@ -2449,7 +2464,7 @@
       <c r="E57" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F57" s="33" t="s">
+      <c r="F57" s="30" t="s">
         <v>36</v>
       </c>
       <c r="G57" s="14">
@@ -2461,14 +2476,14 @@
       <c r="A58" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B58" s="31"/>
+      <c r="B58" s="32"/>
       <c r="C58" s="3">
         <f>1440+560</f>
         <v>2000</v>
       </c>
       <c r="D58" s="3"/>
       <c r="E58" s="9"/>
-      <c r="F58" s="33"/>
+      <c r="F58" s="30"/>
       <c r="G58" s="16">
         <v>2000</v>
       </c>
@@ -2478,7 +2493,7 @@
       <c r="A59" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B59" s="32"/>
+      <c r="B59" s="33"/>
       <c r="C59" s="12">
         <f>C58-C57</f>
         <v>800</v>
@@ -2490,7 +2505,7 @@
       <c r="E59" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F59" s="33"/>
+      <c r="F59" s="30"/>
       <c r="G59" s="15">
         <f>G58-G57</f>
         <v>800</v>
@@ -2503,7 +2518,7 @@
       <c r="A60" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B60" s="30" t="s">
+      <c r="B60" s="31" t="s">
         <v>34</v>
       </c>
       <c r="C60" s="20">
@@ -2516,7 +2531,7 @@
       <c r="E60" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F60" s="33" t="s">
+      <c r="F60" s="30" t="s">
         <v>47</v>
       </c>
       <c r="G60" s="14">
@@ -2528,14 +2543,14 @@
       <c r="A61" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B61" s="31"/>
+      <c r="B61" s="32"/>
       <c r="C61" s="20">
         <f>2000+900</f>
         <v>2900</v>
       </c>
       <c r="D61" s="20"/>
       <c r="E61" s="9"/>
-      <c r="F61" s="33"/>
+      <c r="F61" s="30"/>
       <c r="G61" s="16">
         <v>2900</v>
       </c>
@@ -2545,7 +2560,7 @@
       <c r="A62" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B62" s="32"/>
+      <c r="B62" s="33"/>
       <c r="C62" s="12">
         <f>C61-C60</f>
         <v>1200</v>
@@ -2557,7 +2572,7 @@
       <c r="E62" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F62" s="33"/>
+      <c r="F62" s="30"/>
       <c r="G62" s="15">
         <f>G61-G60</f>
         <v>1100</v>
@@ -2570,7 +2585,7 @@
       <c r="A63" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B63" s="30" t="s">
+      <c r="B63" s="31" t="s">
         <v>34</v>
       </c>
       <c r="C63" s="6">
@@ -2583,7 +2598,7 @@
       <c r="E63" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F63" s="33" t="s">
+      <c r="F63" s="30" t="s">
         <v>46</v>
       </c>
       <c r="G63" s="14">
@@ -2595,14 +2610,14 @@
       <c r="A64" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B64" s="31"/>
+      <c r="B64" s="32"/>
       <c r="C64" s="3">
         <f>2000+1600</f>
         <v>3600</v>
       </c>
       <c r="D64" s="3"/>
       <c r="E64" s="9"/>
-      <c r="F64" s="33"/>
+      <c r="F64" s="30"/>
       <c r="G64" s="16">
         <v>4200</v>
       </c>
@@ -2612,7 +2627,7 @@
       <c r="A65" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B65" s="32"/>
+      <c r="B65" s="33"/>
       <c r="C65" s="12">
         <f>C64-C63</f>
         <v>1600</v>
@@ -2624,7 +2639,7 @@
       <c r="E65" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F65" s="33"/>
+      <c r="F65" s="30"/>
       <c r="G65" s="15">
         <f>G64-G63</f>
         <v>1800</v>
@@ -2651,7 +2666,7 @@
       <c r="A67" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B67" s="30" t="s">
+      <c r="B67" s="31" t="s">
         <v>37</v>
       </c>
       <c r="C67" s="6">
@@ -2663,7 +2678,7 @@
       <c r="E67" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F67" s="33" t="s">
+      <c r="F67" s="30" t="s">
         <v>60</v>
       </c>
       <c r="G67" s="14">
@@ -2675,13 +2690,13 @@
       <c r="A68" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B68" s="31"/>
+      <c r="B68" s="32"/>
       <c r="C68" s="3">
         <v>1200</v>
       </c>
       <c r="D68" s="3"/>
       <c r="E68" s="9"/>
-      <c r="F68" s="33"/>
+      <c r="F68" s="30"/>
       <c r="G68" s="16">
         <v>1200</v>
       </c>
@@ -2691,7 +2706,7 @@
       <c r="A69" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B69" s="32"/>
+      <c r="B69" s="33"/>
       <c r="C69" s="12">
         <f>C68-C67</f>
         <v>600</v>
@@ -2703,7 +2718,7 @@
       <c r="E69" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F69" s="33"/>
+      <c r="F69" s="30"/>
       <c r="G69" s="15">
         <f>G68-G67</f>
         <v>600</v>
@@ -2716,7 +2731,7 @@
       <c r="A70" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B70" s="30" t="s">
+      <c r="B70" s="31" t="s">
         <v>37</v>
       </c>
       <c r="C70" s="6">
@@ -2729,7 +2744,7 @@
       <c r="E70" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F70" s="33" t="s">
+      <c r="F70" s="30" t="s">
         <v>61</v>
       </c>
       <c r="G70" s="14">
@@ -2741,14 +2756,14 @@
       <c r="A71" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B71" s="31"/>
+      <c r="B71" s="32"/>
       <c r="C71" s="3">
         <f>1605+405</f>
         <v>2010</v>
       </c>
       <c r="D71" s="3"/>
       <c r="E71" s="9"/>
-      <c r="F71" s="33"/>
+      <c r="F71" s="30"/>
       <c r="G71" s="16">
         <v>2000</v>
       </c>
@@ -2758,7 +2773,7 @@
       <c r="A72" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B72" s="32"/>
+      <c r="B72" s="33"/>
       <c r="C72" s="12">
         <f>C71-C70</f>
         <v>810</v>
@@ -2770,7 +2785,7 @@
       <c r="E72" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F72" s="33"/>
+      <c r="F72" s="30"/>
       <c r="G72" s="15">
         <f>G71-G70</f>
         <v>800</v>
@@ -2783,7 +2798,7 @@
       <c r="A73" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B73" s="30" t="s">
+      <c r="B73" s="31" t="s">
         <v>37</v>
       </c>
       <c r="C73" s="6">
@@ -2796,7 +2811,7 @@
       <c r="E73" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F73" s="33" t="s">
+      <c r="F73" s="30" t="s">
         <v>62</v>
       </c>
       <c r="G73" s="14">
@@ -2808,14 +2823,14 @@
       <c r="A74" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B74" s="31"/>
+      <c r="B74" s="32"/>
       <c r="C74" s="20">
         <f>1605+900</f>
         <v>2505</v>
       </c>
       <c r="D74" s="20"/>
       <c r="E74" s="9"/>
-      <c r="F74" s="33"/>
+      <c r="F74" s="30"/>
       <c r="G74" s="16">
         <v>2900</v>
       </c>
@@ -2825,7 +2840,7 @@
       <c r="A75" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B75" s="32"/>
+      <c r="B75" s="33"/>
       <c r="C75" s="12">
         <f>C74-C73</f>
         <v>1005</v>
@@ -2837,7 +2852,7 @@
       <c r="E75" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F75" s="33"/>
+      <c r="F75" s="30"/>
       <c r="G75" s="15">
         <f>G74-G73</f>
         <v>1100</v>
@@ -2850,7 +2865,7 @@
       <c r="A76" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B76" s="30" t="s">
+      <c r="B76" s="31" t="s">
         <v>37</v>
       </c>
       <c r="C76" s="6">
@@ -2863,7 +2878,7 @@
       <c r="E76" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F76" s="33" t="s">
+      <c r="F76" s="30" t="s">
         <v>63</v>
       </c>
       <c r="G76" s="14">
@@ -2875,14 +2890,14 @@
       <c r="A77" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B77" s="31"/>
+      <c r="B77" s="32"/>
       <c r="C77" s="20">
         <f>3300+900</f>
         <v>4200</v>
       </c>
       <c r="D77" s="3"/>
       <c r="E77" s="9"/>
-      <c r="F77" s="33"/>
+      <c r="F77" s="30"/>
       <c r="G77" s="16">
         <v>4200</v>
       </c>
@@ -2892,7 +2907,7 @@
       <c r="A78" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B78" s="32"/>
+      <c r="B78" s="33"/>
       <c r="C78" s="12">
         <f>C77-C76</f>
         <v>1890</v>
@@ -2904,7 +2919,7 @@
       <c r="E78" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F78" s="33"/>
+      <c r="F78" s="30"/>
       <c r="G78" s="15">
         <f>G77-G76</f>
         <v>1800</v>
@@ -3968,36 +3983,256 @@
         <v>#VALUE!</v>
       </c>
     </row>
+    <row r="136" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B136" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F136" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H136" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A137" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B137" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="C137" s="6">
+        <v>0</v>
+      </c>
+      <c r="D137" s="6">
+        <v>2500</v>
+      </c>
+      <c r="E137" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="F137" s="29" t="s">
+        <v>74</v>
+      </c>
+      <c r="G137" s="14"/>
+      <c r="H137" s="17"/>
+    </row>
+    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A138" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B138" s="20"/>
+      <c r="C138" s="3">
+        <v>500</v>
+      </c>
+      <c r="D138" s="3"/>
+      <c r="E138" s="9"/>
+      <c r="F138" s="29"/>
+      <c r="G138" s="16"/>
+      <c r="H138" s="18"/>
+    </row>
+    <row r="139" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A139" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B139" s="22"/>
+      <c r="C139" s="12">
+        <f>C138-C137</f>
+        <v>500</v>
+      </c>
+      <c r="D139" s="12">
+        <f>C139/D137</f>
+        <v>0.2</v>
+      </c>
+      <c r="E139" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="F139" s="29"/>
+      <c r="G139" s="15"/>
+      <c r="H139" s="19" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A140" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B140" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="C140" s="6">
+        <v>200</v>
+      </c>
+      <c r="D140" s="6">
+        <v>2500</v>
+      </c>
+      <c r="E140" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="F140" s="29" t="s">
+        <v>75</v>
+      </c>
+      <c r="G140" s="14"/>
+      <c r="H140" s="17"/>
+    </row>
+    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A141" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B141" s="20"/>
+      <c r="C141" s="20">
+        <v>900</v>
+      </c>
+      <c r="D141" s="20"/>
+      <c r="E141" s="9"/>
+      <c r="F141" s="29"/>
+      <c r="G141" s="16"/>
+      <c r="H141" s="18"/>
+    </row>
+    <row r="142" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A142" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B142" s="22"/>
+      <c r="C142" s="12">
+        <f>C141-C140</f>
+        <v>700</v>
+      </c>
+      <c r="D142" s="12">
+        <f>C142/D140</f>
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="E142" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="F142" s="29"/>
+      <c r="G142" s="15"/>
+      <c r="H142" s="19" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A143" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B143" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="C143" s="6">
+        <v>500</v>
+      </c>
+      <c r="D143" s="6">
+        <v>2500</v>
+      </c>
+      <c r="E143" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="F143" s="29" t="s">
+        <v>76</v>
+      </c>
+      <c r="G143" s="14"/>
+      <c r="H143" s="17"/>
+    </row>
+    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A144" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B144" s="20"/>
+      <c r="C144" s="20">
+        <v>1300</v>
+      </c>
+      <c r="D144" s="20"/>
+      <c r="E144" s="9"/>
+      <c r="F144" s="29"/>
+      <c r="G144" s="16"/>
+      <c r="H144" s="18"/>
+    </row>
+    <row r="145" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A145" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B145" s="22"/>
+      <c r="C145" s="12">
+        <f>C144-C143</f>
+        <v>800</v>
+      </c>
+      <c r="D145" s="12">
+        <f>C145/D143</f>
+        <v>0.32</v>
+      </c>
+      <c r="E145" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="F145" s="29"/>
+      <c r="G145" s="15"/>
+      <c r="H145" s="19" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A146" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B146" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="C146" s="6">
+        <f>370+250+240</f>
+        <v>860</v>
+      </c>
+      <c r="D146" s="6">
+        <v>2000</v>
+      </c>
+      <c r="E146" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="F146" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="G146" s="14"/>
+      <c r="H146" s="17"/>
+    </row>
+    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A147" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B147" s="20"/>
+      <c r="C147" s="20">
+        <v>1700</v>
+      </c>
+      <c r="D147" s="3"/>
+      <c r="E147" s="9"/>
+      <c r="F147" s="29"/>
+      <c r="G147" s="16"/>
+      <c r="H147" s="18"/>
+    </row>
+    <row r="148" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A148" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B148" s="22"/>
+      <c r="C148" s="12">
+        <f>C147-C146</f>
+        <v>840</v>
+      </c>
+      <c r="D148" s="12">
+        <f>C148/D146</f>
+        <v>0.42</v>
+      </c>
+      <c r="E148" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="F148" s="29"/>
+      <c r="G148" s="15"/>
+      <c r="H148" s="19" t="s">
+        <v>45</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="44">
-    <mergeCell ref="F37:F39"/>
-    <mergeCell ref="F34:F36"/>
-    <mergeCell ref="N2:N4"/>
-    <mergeCell ref="N5:N7"/>
-    <mergeCell ref="N8:N10"/>
-    <mergeCell ref="N11:N13"/>
-    <mergeCell ref="F31:F33"/>
-    <mergeCell ref="F15:F17"/>
-    <mergeCell ref="F18:F20"/>
-    <mergeCell ref="F24:F26"/>
-    <mergeCell ref="F2:F4"/>
-    <mergeCell ref="F5:F7"/>
-    <mergeCell ref="F8:F10"/>
-    <mergeCell ref="F11:F13"/>
-    <mergeCell ref="F41:F43"/>
-    <mergeCell ref="F44:F46"/>
-    <mergeCell ref="F50:F52"/>
-    <mergeCell ref="F47:F49"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="B44:B46"/>
-    <mergeCell ref="B47:B49"/>
-    <mergeCell ref="B50:B52"/>
-    <mergeCell ref="B54:B56"/>
-    <mergeCell ref="F54:F56"/>
-    <mergeCell ref="B57:B59"/>
-    <mergeCell ref="F57:F59"/>
-    <mergeCell ref="B60:B62"/>
-    <mergeCell ref="F60:F62"/>
+  <mergeCells count="48">
+    <mergeCell ref="F137:F139"/>
+    <mergeCell ref="F140:F142"/>
+    <mergeCell ref="F146:F148"/>
+    <mergeCell ref="F143:F145"/>
     <mergeCell ref="F121:F123"/>
     <mergeCell ref="F124:F126"/>
     <mergeCell ref="F127:F129"/>
@@ -4014,6 +4249,34 @@
     <mergeCell ref="F88:F90"/>
     <mergeCell ref="B76:B78"/>
     <mergeCell ref="F76:F78"/>
+    <mergeCell ref="B54:B56"/>
+    <mergeCell ref="F54:F56"/>
+    <mergeCell ref="B57:B59"/>
+    <mergeCell ref="F57:F59"/>
+    <mergeCell ref="B60:B62"/>
+    <mergeCell ref="F60:F62"/>
+    <mergeCell ref="F41:F43"/>
+    <mergeCell ref="F44:F46"/>
+    <mergeCell ref="F50:F52"/>
+    <mergeCell ref="F47:F49"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="B47:B49"/>
+    <mergeCell ref="B50:B52"/>
+    <mergeCell ref="F37:F39"/>
+    <mergeCell ref="F34:F36"/>
+    <mergeCell ref="N2:N4"/>
+    <mergeCell ref="N5:N7"/>
+    <mergeCell ref="N8:N10"/>
+    <mergeCell ref="N11:N13"/>
+    <mergeCell ref="F31:F33"/>
+    <mergeCell ref="F15:F17"/>
+    <mergeCell ref="F18:F20"/>
+    <mergeCell ref="F24:F26"/>
+    <mergeCell ref="F2:F4"/>
+    <mergeCell ref="F5:F7"/>
+    <mergeCell ref="F8:F10"/>
+    <mergeCell ref="F11:F13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>